<commit_message>
feat: group operation history by change
</commit_message>
<xml_diff>
--- a/docs/数据库表结构.xlsx
+++ b/docs/数据库表结构.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="Rd40198d6f67f44f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="R0239707e36184be2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="R2426dc62deb748b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="Rf4b784e5da244ec2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="R237e65893a06434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R56b778ce8e1f4972"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="R38dbdf9f249c4ed9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="Rdcad48a3d8e94dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R5a2e20d2154a47c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="R43b3fbbea4404882"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="R24a613988c8b4a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Rd03b6ad23d484af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R63f0a904052e4e7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="Ra6082f9ea4f84b70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="Rd30e3fa941b44403"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="R9a66996217124dd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="Rb0748ef8007d49e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="Rdd67fbce6e804a33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="R82eb2f18fc114b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="Re04ccba0fe7c4d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="R7434f07979934eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R60bedb98fa3d4381"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="Rb0e9625dfc6c49e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="Rc4b58edc76b0483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="R25c88550db684b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Rd6c2e05cbc3745d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="Rbb6ede752ec047a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="R24e20227f7e64689"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2799,8 +2799,8 @@
     <x:col min="6" max="6" width="9.852941513061523" style="2" customWidth="1"/>
     <x:col min="7" max="7" width="7.352941036224365" style="2" customWidth="1"/>
     <x:col min="8" max="8" width="6.411764621734619" style="2" customWidth="1"/>
-    <x:col min="9" max="9" width="19.117647171020508" style="2" customWidth="1"/>
-    <x:col min="10" max="10" width="13.970588684082031" style="2" customWidth="1"/>
+    <x:col min="9" max="9" width="34" style="2" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" style="2" hidden="0" customWidth="1"/>
     <x:col min="11" max="16384" width="55.764705657958984" style="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -3103,28 +3103,54 @@
       </x:c>
     </x:row>
     <x:row r="13" s="1" customFormat="1">
-      <x:c r="A13" s="9" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="C13" s="9" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="D13" s="9" t="s">
-        <x:v>90</x:v>
-      </x:c>
+      <x:c r="A13" s="9" t="str">
+        <x:v>操作批次ID</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>operation_id</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="str">
+        <x:v>UUID</x:v>
+      </x:c>
+      <x:c r="D13" s="9"/>
       <x:c r="E13" s="9"/>
       <x:c r="F13" s="9"/>
-      <x:c r="G13" s="9"/>
-      <x:c r="H13" s="9" t="s">
+      <x:c r="G13" s="9" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="str">
+        <x:v>NULL</x:v>
+      </x:c>
+      <x:c r="I13" s="9" t="str">
+        <x:v>550e8400-e29b-41d4-a716-446655440000</x:v>
+      </x:c>
+      <x:c r="J13" s="9" t="str">
+        <x:v>同一次业务操作共享，用于聚合多字段变更。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="B14" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="C14" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D14" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="I13" s="9" t="s">
+      <x:c r="I14" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="J13" s="9" t="s">
+      <x:c r="J14" t="s">
         <x:v>301</x:v>
       </x:c>
     </x:row>
@@ -4489,7 +4515,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R788f66b8ccf94cd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a184306063848ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add unified business attachments
</commit_message>
<xml_diff>
--- a/docs/数据库表结构.xlsx
+++ b/docs/数据库表结构.xlsx
@@ -2,46 +2,47 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="R598066ce45924cd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="Rdd9c21322ae04fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段汇总" sheetId="31" r:id="Rdf73f606624840b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="R9c1908b5c1ad40f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="Rbead0583b0a34b77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="R64edac48469141c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R533a277034614c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="R135a5ed9b44e493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R52c522ba3c754310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="Rb1e653942f2e464d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="Rf4eba98ec4934d35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="R626e2e597fb94408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="R45c5bd7daf0c4019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R032fa11a29a5415e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="R7c4c9e8ddda94d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product" sheetId="15" r:id="Rb8fe5200d2f04769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project" sheetId="16" r:id="Rf437723395a14346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_member" sheetId="17" r:id="R1ec50f03390048d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_requirement" sheetId="18" r:id="R60272b4867ac455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task" sheetId="19" r:id="Rdbabbc26f65341d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task_owner" sheetId="30" r:id="R9ac86962d16e45f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_bug" sheetId="20" r:id="R59af6c2c31dd4c3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract" sheetId="21" r:id="Re283412084f4486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_stage" sheetId="22" r:id="R98315dfe937b4cde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_record" sheetId="23" r:id="R4c8fe06484c9450d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract_attachment" sheetId="24" r:id="Rbf8b40fcd31241e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_stage" sheetId="25" r:id="R8c389d0e09e1432a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item" sheetId="26" r:id="R9c9ad31c92f74875"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item_collabora" sheetId="27" r:id="R4f0cda7b61344b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_adjustment" sheetId="28" r:id="Rb577d4e39e134340"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_delivery_file" sheetId="29" r:id="Rb044f1b8c4184ded"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_client" sheetId="32" r:id="Rce3d660fae8f4a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_audit_log" sheetId="33" r:id="R5fdf1fe74ca84e78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_action_ticket" sheetId="34" r:id="R8d1e1fba1abb4f34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template" sheetId="35" r:id="R922ebf59939b4294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_stage" sheetId="36" r:id="Rd8b54803a16e43a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_item" sheetId="37" r:id="Re794dbf94cee42a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract" sheetId="38" r:id="R109b892c6215466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract_attachment" sheetId="39" r:id="Rd628293a55964965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_scheduled_task_execution" sheetId="40" r:id="R6336962012ac460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="R5000a7eecfbe4481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="R0d254a0a70514fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段汇总" sheetId="31" r:id="Rc6716c3430b74a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="R212e55bf7fd24c6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="Rb5b63bb5eac34717"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="R4a512cfa369c4c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R0f12c807b88a4b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="R6790a607e89f4ef9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R8ba5481a28fc4f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R18ebed75314949dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="R7c66f246d1ad4c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="R9f4b0b09b1044a34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Ra31ea2163cea491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R2e6afab358b14360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="R848f608d8efb4278"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product" sheetId="15" r:id="R3127cff3f47e4f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project" sheetId="16" r:id="Rcc51760466834866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_member" sheetId="17" r:id="Rbb109a6401e4467a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_requirement" sheetId="18" r:id="R0219e179713d4005"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task" sheetId="19" r:id="R206b317edcd64488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_task_owner" sheetId="30" r:id="Rc01e3c2f769f43f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_bug" sheetId="20" r:id="Ra2a1269325ce49dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract" sheetId="21" r:id="R732f72744c1b4bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_stage" sheetId="22" r:id="Rd8258a7ba78f4019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_payment_record" sheetId="23" r:id="Rb5ecc719bbaf4a27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_contract_attachment" sheetId="24" r:id="Rf73cb7a197ad471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_stage" sheetId="25" r:id="Race7eec57b6145aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item" sheetId="26" r:id="R4b00abf9684c44c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_item_collabora" sheetId="27" r:id="Rba9fb8d93c944350"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_adjustment" sheetId="28" r:id="R4ffa7946df074689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_delivery_file" sheetId="29" r:id="R69e1f59bfa5d40fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_client" sheetId="32" r:id="R07ba1c15991f4af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_audit_log" sheetId="33" r:id="R0fcb9ce808c7469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_mcp_action_ticket" sheetId="34" r:id="R70b830c748314ba5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template" sheetId="35" r:id="R42b81986d5284972"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_stage" sheetId="36" r:id="R9019d348fea54bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_project_plan_template_item" sheetId="37" r:id="Rc45cf8c3add346af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract" sheetId="38" r:id="R198ba0b47e944094"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_product_maintenance_contract_attachment" sheetId="39" r:id="R0b42ace4768248ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_scheduled_task_execution" sheetId="40" r:id="R25f318667ac94904"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_business_attachment" sheetId="41" r:id="Rfe883cb351fd46bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2299,7 +2300,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="39">
+  <x:fills count="41">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2489,6 +2490,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFC5E8F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B9BD5"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -2810,7 +2821,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="63">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
@@ -2927,6 +2938,38 @@
     <x:xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="25" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="39" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="40" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="40" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="40" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="40" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="50">
@@ -8136,10 +8179,24 @@
         <x:v>通用定时任务幂等、执行状态、重试和结果记录。</x:v>
       </x:c>
     </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>需求、项目、任务、BUG、运维工单的 OSS 附件元数据。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0db8c70f3a894476"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb4ad46dd0034b54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28784,6 +28841,540 @@
         <x:v>NOT NULL</x:v>
       </x:c>
     </x:row>
+    <x:row r="453">
+      <x:c r="A453" t="n">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="B453" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C453" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D453" t="str">
+        <x:v>主键ID</x:v>
+      </x:c>
+      <x:c r="E453" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="F453" t="str">
+        <x:v>BIGSERIAL</x:v>
+      </x:c>
+      <x:c r="G453" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H453" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I453"/>
+      <x:c r="J453" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K453" t="str">
+        <x:v>自增</x:v>
+      </x:c>
+      <x:c r="L453" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M453" t="str">
+        <x:v>附件主键。</x:v>
+      </x:c>
+      <x:c r="N453" t="str">
+        <x:v>PRIMARY KEY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="454">
+      <x:c r="A454" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="B454" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C454" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D454" t="str">
+        <x:v>业务类型</x:v>
+      </x:c>
+      <x:c r="E454" t="str">
+        <x:v>business_type</x:v>
+      </x:c>
+      <x:c r="F454" t="str">
+        <x:v>VARCHAR(30)</x:v>
+      </x:c>
+      <x:c r="G454" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H454"/>
+      <x:c r="I454"/>
+      <x:c r="J454" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K454"/>
+      <x:c r="L454" t="str">
+        <x:v>task</x:v>
+      </x:c>
+      <x:c r="M454" t="str">
+        <x:v>requirement、project、task、bug 或 work_order。</x:v>
+      </x:c>
+      <x:c r="N454" t="str">
+        <x:v>CHECK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="455">
+      <x:c r="A455" t="n">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="B455" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C455" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D455" t="str">
+        <x:v>业务记录ID</x:v>
+      </x:c>
+      <x:c r="E455" t="str">
+        <x:v>business_id</x:v>
+      </x:c>
+      <x:c r="F455" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G455" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H455"/>
+      <x:c r="I455"/>
+      <x:c r="J455" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K455"/>
+      <x:c r="L455" t="str">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="M455" t="str">
+        <x:v>多态关联的业务记录主键，不设置物理外键。</x:v>
+      </x:c>
+      <x:c r="N455" t="str">
+        <x:v>NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="456">
+      <x:c r="A456" t="n">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="B456" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C456" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D456" t="str">
+        <x:v>原文件名</x:v>
+      </x:c>
+      <x:c r="E456" t="str">
+        <x:v>original_name</x:v>
+      </x:c>
+      <x:c r="F456" t="str">
+        <x:v>VARCHAR(255)</x:v>
+      </x:c>
+      <x:c r="G456" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H456"/>
+      <x:c r="I456"/>
+      <x:c r="J456"/>
+      <x:c r="K456"/>
+      <x:c r="L456" t="str">
+        <x:v>需求说明书.pdf</x:v>
+      </x:c>
+      <x:c r="M456" t="str">
+        <x:v>上传时的原文件名。</x:v>
+      </x:c>
+      <x:c r="N456" t="str">
+        <x:v>NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="457">
+      <x:c r="A457" t="n">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="B457" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C457" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D457" t="str">
+        <x:v>文件类型</x:v>
+      </x:c>
+      <x:c r="E457" t="str">
+        <x:v>mime_type</x:v>
+      </x:c>
+      <x:c r="F457" t="str">
+        <x:v>VARCHAR(150)</x:v>
+      </x:c>
+      <x:c r="G457" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H457"/>
+      <x:c r="I457"/>
+      <x:c r="J457"/>
+      <x:c r="K457"/>
+      <x:c r="L457" t="str">
+        <x:v>application/pdf</x:v>
+      </x:c>
+      <x:c r="M457" t="str">
+        <x:v>文件 MIME 类型。</x:v>
+      </x:c>
+      <x:c r="N457" t="str">
+        <x:v>NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="458">
+      <x:c r="A458" t="n">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="B458" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C458" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D458" t="str">
+        <x:v>文件大小</x:v>
+      </x:c>
+      <x:c r="E458" t="str">
+        <x:v>file_size</x:v>
+      </x:c>
+      <x:c r="F458" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G458" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H458"/>
+      <x:c r="I458"/>
+      <x:c r="J458"/>
+      <x:c r="K458"/>
+      <x:c r="L458" t="str">
+        <x:v>102400</x:v>
+      </x:c>
+      <x:c r="M458" t="str">
+        <x:v>单位字节；大于 0 且不超过 20971520。</x:v>
+      </x:c>
+      <x:c r="N458" t="str">
+        <x:v>CHECK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="459">
+      <x:c r="A459" t="n">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="B459" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C459" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D459" t="str">
+        <x:v>OSS存储键</x:v>
+      </x:c>
+      <x:c r="E459" t="str">
+        <x:v>storage_key</x:v>
+      </x:c>
+      <x:c r="F459" t="str">
+        <x:v>VARCHAR(255)</x:v>
+      </x:c>
+      <x:c r="G459" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H459" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I459"/>
+      <x:c r="J459" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K459"/>
+      <x:c r="L459" t="str">
+        <x:v>business/task/80/file.pdf</x:v>
+      </x:c>
+      <x:c r="M459" t="str">
+        <x:v>OSS 文件路径。</x:v>
+      </x:c>
+      <x:c r="N459" t="str">
+        <x:v>UNIQUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="460">
+      <x:c r="A460" t="n">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="B460" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C460" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D460" t="str">
+        <x:v>OSS响应</x:v>
+      </x:c>
+      <x:c r="E460" t="str">
+        <x:v>oss_response</x:v>
+      </x:c>
+      <x:c r="F460" t="str">
+        <x:v>JSONB</x:v>
+      </x:c>
+      <x:c r="G460" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H460"/>
+      <x:c r="I460"/>
+      <x:c r="J460"/>
+      <x:c r="K460"/>
+      <x:c r="L460" t="str">
+        <x:v>{"code":100,"msg":"success"}</x:v>
+      </x:c>
+      <x:c r="M460" t="str">
+        <x:v>OSS 上传接口返回的完整 JSON。</x:v>
+      </x:c>
+      <x:c r="N460" t="str">
+        <x:v>NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="461">
+      <x:c r="A461" t="n">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="B461" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C461" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D461" t="str">
+        <x:v>排序号</x:v>
+      </x:c>
+      <x:c r="E461" t="str">
+        <x:v>sort_order</x:v>
+      </x:c>
+      <x:c r="F461" t="str">
+        <x:v>INTEGER</x:v>
+      </x:c>
+      <x:c r="G461" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H461"/>
+      <x:c r="I461"/>
+      <x:c r="J461" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K461" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L461" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M461" t="str">
+        <x:v>同一业务记录附件的显示顺序。</x:v>
+      </x:c>
+      <x:c r="N461" t="str">
+        <x:v>NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="462">
+      <x:c r="A462" t="n">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="B462" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C462" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D462" t="str">
+        <x:v>创建人ID</x:v>
+      </x:c>
+      <x:c r="E462" t="str">
+        <x:v>creator_id</x:v>
+      </x:c>
+      <x:c r="F462" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G462"/>
+      <x:c r="H462"/>
+      <x:c r="I462" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="J462"/>
+      <x:c r="K462" t="str">
+        <x:v>NULL</x:v>
+      </x:c>
+      <x:c r="L462" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M462" t="str">
+        <x:v>记录上传人。</x:v>
+      </x:c>
+      <x:c r="N462" t="str">
+        <x:v>ON DELETE SET NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="463">
+      <x:c r="A463" t="n">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="B463" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C463" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D463" t="str">
+        <x:v>更新人ID</x:v>
+      </x:c>
+      <x:c r="E463" t="str">
+        <x:v>updater_id</x:v>
+      </x:c>
+      <x:c r="F463" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="G463"/>
+      <x:c r="H463"/>
+      <x:c r="I463" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="J463"/>
+      <x:c r="K463" t="str">
+        <x:v>NULL</x:v>
+      </x:c>
+      <x:c r="L463" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M463" t="str">
+        <x:v>记录最后更新人。</x:v>
+      </x:c>
+      <x:c r="N463" t="str">
+        <x:v>ON DELETE SET NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="464">
+      <x:c r="A464" t="n">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="B464" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C464" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D464" t="str">
+        <x:v>删除标记</x:v>
+      </x:c>
+      <x:c r="E464" t="str">
+        <x:v>is_deleted</x:v>
+      </x:c>
+      <x:c r="F464" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="G464" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H464"/>
+      <x:c r="I464"/>
+      <x:c r="J464" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="K464" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L464" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M464" t="str">
+        <x:v>0 正常，1 删除。</x:v>
+      </x:c>
+      <x:c r="N464" t="str">
+        <x:v>CHECK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="465">
+      <x:c r="A465" t="n">
+        <x:v>461</x:v>
+      </x:c>
+      <x:c r="B465" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C465" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D465" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="E465" t="str">
+        <x:v>created_at</x:v>
+      </x:c>
+      <x:c r="F465" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="G465" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H465"/>
+      <x:c r="I465"/>
+      <x:c r="J465"/>
+      <x:c r="K465" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="L465" t="str">
+        <x:v>2026-08-19 10:00:00</x:v>
+      </x:c>
+      <x:c r="M465" t="str">
+        <x:v>记录上传时间。</x:v>
+      </x:c>
+      <x:c r="N465" t="str">
+        <x:v>NOT NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="466">
+      <x:c r="A466" t="n">
+        <x:v>462</x:v>
+      </x:c>
+      <x:c r="B466" t="str">
+        <x:v>pms_business_attachment</x:v>
+      </x:c>
+      <x:c r="C466" t="str">
+        <x:v>通用业务附件表</x:v>
+      </x:c>
+      <x:c r="D466" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="E466" t="str">
+        <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="F466" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="G466" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H466"/>
+      <x:c r="I466"/>
+      <x:c r="J466"/>
+      <x:c r="K466" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="L466" t="str">
+        <x:v>2026-08-19 10:00:00</x:v>
+      </x:c>
+      <x:c r="M466" t="str">
+        <x:v>记录最后更新时间。</x:v>
+      </x:c>
+      <x:c r="N466" t="str">
+        <x:v>NOT NULL</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
@@ -28791,7 +29382,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd93456aa2b41450a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf906115616944d4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29844,7 +30435,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36e13a02e6434a8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4683fc36d0a14fe6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30423,7 +31014,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62afc60774d440a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7869814ef0984dee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30834,7 +31425,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R250f19950842412e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59ab38faf32542d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31121,7 +31712,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cfa3d3255294c21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4112073f8304b78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31382,7 +31973,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4803bc6d4d6a408f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcde7d7b1a56b4657"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31695,7 +32286,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8c9ddf630ee4bc3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R380c3df128e64975"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33485,6 +34076,442 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="47.779998779296875" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="51" t="str">
+        <x:v>pms_business_attachment（通用业务附件表）</x:v>
+      </x:c>
+      <x:c r="B1" s="51"/>
+      <x:c r="C1" s="51"/>
+      <x:c r="D1" s="51"/>
+      <x:c r="E1" s="51"/>
+      <x:c r="F1" s="51"/>
+      <x:c r="G1" s="51"/>
+      <x:c r="H1" s="51"/>
+      <x:c r="I1" s="51"/>
+      <x:c r="J1" s="51"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="57" t="str">
+        <x:v>中文字段名</x:v>
+      </x:c>
+      <x:c r="B2" s="57" t="str">
+        <x:v>技术字段名</x:v>
+      </x:c>
+      <x:c r="C2" s="57" t="str">
+        <x:v>数据类型</x:v>
+      </x:c>
+      <x:c r="D2" s="57" t="str">
+        <x:v>必填</x:v>
+      </x:c>
+      <x:c r="E2" s="57" t="str">
+        <x:v>是否唯一</x:v>
+      </x:c>
+      <x:c r="F2" s="57" t="str">
+        <x:v>关联引用</x:v>
+      </x:c>
+      <x:c r="G2" s="57" t="str">
+        <x:v>是否索引</x:v>
+      </x:c>
+      <x:c r="H2" s="57" t="str">
+        <x:v>默认值</x:v>
+      </x:c>
+      <x:c r="I2" s="57" t="str">
+        <x:v>示例</x:v>
+      </x:c>
+      <x:c r="J2" s="57" t="str">
+        <x:v>字段说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="62" t="str">
+        <x:v>主键ID</x:v>
+      </x:c>
+      <x:c r="B3" s="62" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C3" s="62" t="str">
+        <x:v>BIGSERIAL</x:v>
+      </x:c>
+      <x:c r="D3" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E3" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F3" s="62"/>
+      <x:c r="G3" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H3" s="62" t="str">
+        <x:v>自增</x:v>
+      </x:c>
+      <x:c r="I3" s="62" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J3" s="62" t="str">
+        <x:v>附件主键。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="62" t="str">
+        <x:v>业务类型</x:v>
+      </x:c>
+      <x:c r="B4" s="62" t="str">
+        <x:v>business_type</x:v>
+      </x:c>
+      <x:c r="C4" s="62" t="str">
+        <x:v>VARCHAR(30)</x:v>
+      </x:c>
+      <x:c r="D4" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E4" s="62"/>
+      <x:c r="F4" s="62"/>
+      <x:c r="G4" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H4" s="62"/>
+      <x:c r="I4" s="62" t="str">
+        <x:v>task</x:v>
+      </x:c>
+      <x:c r="J4" s="62" t="str">
+        <x:v>requirement、project、task、bug 或 work_order。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="62" t="str">
+        <x:v>业务记录ID</x:v>
+      </x:c>
+      <x:c r="B5" s="62" t="str">
+        <x:v>business_id</x:v>
+      </x:c>
+      <x:c r="C5" s="62" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D5" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E5" s="62"/>
+      <x:c r="F5" s="62"/>
+      <x:c r="G5" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H5" s="62"/>
+      <x:c r="I5" s="62" t="str">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="J5" s="62" t="str">
+        <x:v>多态关联的业务记录主键，不设置物理外键。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="62" t="str">
+        <x:v>原文件名</x:v>
+      </x:c>
+      <x:c r="B6" s="62" t="str">
+        <x:v>original_name</x:v>
+      </x:c>
+      <x:c r="C6" s="62" t="str">
+        <x:v>VARCHAR(255)</x:v>
+      </x:c>
+      <x:c r="D6" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E6" s="62"/>
+      <x:c r="F6" s="62"/>
+      <x:c r="G6" s="62"/>
+      <x:c r="H6" s="62"/>
+      <x:c r="I6" s="62" t="str">
+        <x:v>需求说明书.pdf</x:v>
+      </x:c>
+      <x:c r="J6" s="62" t="str">
+        <x:v>上传时的原文件名。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="62" t="str">
+        <x:v>文件类型</x:v>
+      </x:c>
+      <x:c r="B7" s="62" t="str">
+        <x:v>mime_type</x:v>
+      </x:c>
+      <x:c r="C7" s="62" t="str">
+        <x:v>VARCHAR(150)</x:v>
+      </x:c>
+      <x:c r="D7" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E7" s="62"/>
+      <x:c r="F7" s="62"/>
+      <x:c r="G7" s="62"/>
+      <x:c r="H7" s="62"/>
+      <x:c r="I7" s="62" t="str">
+        <x:v>application/pdf</x:v>
+      </x:c>
+      <x:c r="J7" s="62" t="str">
+        <x:v>文件 MIME 类型。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="62" t="str">
+        <x:v>文件大小</x:v>
+      </x:c>
+      <x:c r="B8" s="62" t="str">
+        <x:v>file_size</x:v>
+      </x:c>
+      <x:c r="C8" s="62" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D8" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E8" s="62"/>
+      <x:c r="F8" s="62"/>
+      <x:c r="G8" s="62"/>
+      <x:c r="H8" s="62"/>
+      <x:c r="I8" s="62" t="str">
+        <x:v>102400</x:v>
+      </x:c>
+      <x:c r="J8" s="62" t="str">
+        <x:v>单位字节；大于 0 且不超过 20971520。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="62" t="str">
+        <x:v>OSS存储键</x:v>
+      </x:c>
+      <x:c r="B9" s="62" t="str">
+        <x:v>storage_key</x:v>
+      </x:c>
+      <x:c r="C9" s="62" t="str">
+        <x:v>VARCHAR(255)</x:v>
+      </x:c>
+      <x:c r="D9" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E9" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F9" s="62"/>
+      <x:c r="G9" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H9" s="62"/>
+      <x:c r="I9" s="62" t="str">
+        <x:v>business/task/80/file.pdf</x:v>
+      </x:c>
+      <x:c r="J9" s="62" t="str">
+        <x:v>OSS 文件路径。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="62" t="str">
+        <x:v>OSS响应</x:v>
+      </x:c>
+      <x:c r="B10" s="62" t="str">
+        <x:v>oss_response</x:v>
+      </x:c>
+      <x:c r="C10" s="62" t="str">
+        <x:v>JSONB</x:v>
+      </x:c>
+      <x:c r="D10" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E10" s="62"/>
+      <x:c r="F10" s="62"/>
+      <x:c r="G10" s="62"/>
+      <x:c r="H10" s="62"/>
+      <x:c r="I10" s="62" t="str">
+        <x:v>{"code":100,"msg":"success"}</x:v>
+      </x:c>
+      <x:c r="J10" s="62" t="str">
+        <x:v>OSS 上传接口返回的完整 JSON。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="62" t="str">
+        <x:v>排序号</x:v>
+      </x:c>
+      <x:c r="B11" s="62" t="str">
+        <x:v>sort_order</x:v>
+      </x:c>
+      <x:c r="C11" s="62" t="str">
+        <x:v>INTEGER</x:v>
+      </x:c>
+      <x:c r="D11" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E11" s="62"/>
+      <x:c r="F11" s="62"/>
+      <x:c r="G11" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H11" s="62" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="62" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="62" t="str">
+        <x:v>同一业务记录附件的显示顺序。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="62" t="str">
+        <x:v>创建人ID</x:v>
+      </x:c>
+      <x:c r="B12" s="62" t="str">
+        <x:v>creator_id</x:v>
+      </x:c>
+      <x:c r="C12" s="62" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D12" s="62"/>
+      <x:c r="E12" s="62"/>
+      <x:c r="F12" s="62" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="G12" s="62"/>
+      <x:c r="H12" s="62" t="str">
+        <x:v>NULL</x:v>
+      </x:c>
+      <x:c r="I12" s="62" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J12" s="62" t="str">
+        <x:v>记录上传人。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="62" t="str">
+        <x:v>更新人ID</x:v>
+      </x:c>
+      <x:c r="B13" s="62" t="str">
+        <x:v>updater_id</x:v>
+      </x:c>
+      <x:c r="C13" s="62" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D13" s="62"/>
+      <x:c r="E13" s="62"/>
+      <x:c r="F13" s="62" t="str">
+        <x:v>pms_user.id</x:v>
+      </x:c>
+      <x:c r="G13" s="62"/>
+      <x:c r="H13" s="62" t="str">
+        <x:v>NULL</x:v>
+      </x:c>
+      <x:c r="I13" s="62" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J13" s="62" t="str">
+        <x:v>记录最后更新人。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="62" t="str">
+        <x:v>删除标记</x:v>
+      </x:c>
+      <x:c r="B14" s="62" t="str">
+        <x:v>is_deleted</x:v>
+      </x:c>
+      <x:c r="C14" s="62" t="str">
+        <x:v>SMALLINT</x:v>
+      </x:c>
+      <x:c r="D14" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E14" s="62"/>
+      <x:c r="F14" s="62"/>
+      <x:c r="G14" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H14" s="62" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" s="62" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J14" s="62" t="str">
+        <x:v>0 正常，1 删除。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="62" t="str">
+        <x:v>创建时间</x:v>
+      </x:c>
+      <x:c r="B15" s="62" t="str">
+        <x:v>created_at</x:v>
+      </x:c>
+      <x:c r="C15" s="62" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="D15" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E15" s="62"/>
+      <x:c r="F15" s="62"/>
+      <x:c r="G15" s="62"/>
+      <x:c r="H15" s="62" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="I15" s="62" t="str">
+        <x:v>2026-08-19 10:00:00</x:v>
+      </x:c>
+      <x:c r="J15" s="62" t="str">
+        <x:v>记录上传时间。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="62" t="str">
+        <x:v>更新时间</x:v>
+      </x:c>
+      <x:c r="B16" s="62" t="str">
+        <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="C16" s="62" t="str">
+        <x:v>TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="D16" s="62" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="E16" s="62"/>
+      <x:c r="F16" s="62"/>
+      <x:c r="G16" s="62"/>
+      <x:c r="H16" s="62" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+      <x:c r="I16" s="62" t="str">
+        <x:v>2026-08-19 10:00:00</x:v>
+      </x:c>
+      <x:c r="J16" s="62" t="str">
+        <x:v>记录最后更新时间。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultColWidth="9" defaultRowHeight="16.799999237060547"/>

</xml_diff>